<commit_message>
Update Zuimeng attribute stats from latest table
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,35 +590,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>抹小茶</t>
+          <t>犹大刃舞</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>147757844</v>
+        <v>145308669</v>
       </c>
       <c r="D5" t="n">
-        <v>31.08</v>
+        <v>31.72</v>
       </c>
       <c r="E5" t="n">
-        <v>1485</v>
+        <v>1678</v>
       </c>
       <c r="F5" t="n">
-        <v>1126.3</v>
+        <v>1219</v>
       </c>
       <c r="G5" t="n">
-        <v>1180</v>
+        <v>1312</v>
       </c>
       <c r="H5" t="n">
-        <v>933</v>
+        <v>1042</v>
       </c>
       <c r="I5" t="n">
-        <v>908</v>
+        <v>1021</v>
       </c>
       <c r="J5" t="n">
-        <v>978</v>
+        <v>1123</v>
       </c>
       <c r="K5" t="n">
-        <v>6610</v>
+        <v>7395</v>
       </c>
     </row>
     <row r="6">
@@ -664,35 +664,35 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>犹大刃舞</t>
+          <t>点点点的小号</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>145308669</v>
+        <v>131182828</v>
       </c>
       <c r="D7" t="n">
-        <v>31.72</v>
+        <v>31.08</v>
       </c>
       <c r="E7" t="n">
-        <v>1678</v>
+        <v>1484</v>
       </c>
       <c r="F7" t="n">
-        <v>1219</v>
+        <v>1166</v>
       </c>
       <c r="G7" t="n">
-        <v>1312</v>
+        <v>1168</v>
       </c>
       <c r="H7" t="n">
-        <v>1042</v>
+        <v>1029</v>
       </c>
       <c r="I7" t="n">
-        <v>1021</v>
+        <v>973</v>
       </c>
       <c r="J7" t="n">
-        <v>1123</v>
+        <v>1045</v>
       </c>
       <c r="K7" t="n">
-        <v>7395</v>
+        <v>6865</v>
       </c>
     </row>
     <row r="8">
@@ -738,35 +738,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>事后清晨001</t>
+          <t>吉多多</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>136247069</v>
+        <v>132970854</v>
       </c>
       <c r="D9" t="n">
         <v>31.08</v>
       </c>
       <c r="E9" t="n">
-        <v>1414</v>
+        <v>1313</v>
       </c>
       <c r="F9" t="n">
-        <v>1117</v>
+        <v>1150</v>
       </c>
       <c r="G9" t="n">
-        <v>1141</v>
+        <v>1168</v>
       </c>
       <c r="H9" t="n">
-        <v>1024</v>
+        <v>1017</v>
       </c>
       <c r="I9" t="n">
-        <v>750</v>
+        <v>1001</v>
       </c>
       <c r="J9" t="n">
-        <v>945</v>
+        <v>1107</v>
       </c>
       <c r="K9" t="n">
-        <v>6391</v>
+        <v>6756</v>
       </c>
     </row>
     <row r="10">
@@ -775,35 +775,35 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>吉多多</t>
+          <t>慢下来</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>132970854</v>
+        <v>130572370</v>
       </c>
       <c r="D10" t="n">
         <v>31.08</v>
       </c>
       <c r="E10" t="n">
-        <v>1301</v>
+        <v>1366</v>
       </c>
       <c r="F10" t="n">
-        <v>1111</v>
+        <v>1133</v>
       </c>
       <c r="G10" t="n">
-        <v>1168</v>
+        <v>1255</v>
       </c>
       <c r="H10" t="n">
+        <v>1006</v>
+      </c>
+      <c r="I10" t="n">
         <v>974</v>
       </c>
-      <c r="I10" t="n">
-        <v>958</v>
-      </c>
       <c r="J10" t="n">
-        <v>1097</v>
+        <v>969</v>
       </c>
       <c r="K10" t="n">
-        <v>6609</v>
+        <v>6703</v>
       </c>
     </row>
     <row r="11">
@@ -812,35 +812,35 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>点点点的小号</t>
+          <t>抹小茶</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>131182828</v>
+        <v>147757844</v>
       </c>
       <c r="D11" t="n">
         <v>31.08</v>
       </c>
       <c r="E11" t="n">
-        <v>1484</v>
+        <v>1485</v>
       </c>
       <c r="F11" t="n">
-        <v>1166</v>
+        <v>1126.3</v>
       </c>
       <c r="G11" t="n">
-        <v>1168</v>
+        <v>1180</v>
       </c>
       <c r="H11" t="n">
-        <v>1029</v>
+        <v>933</v>
       </c>
       <c r="I11" t="n">
-        <v>973</v>
+        <v>908</v>
       </c>
       <c r="J11" t="n">
-        <v>1045</v>
+        <v>978</v>
       </c>
       <c r="K11" t="n">
-        <v>6865</v>
+        <v>6610</v>
       </c>
     </row>
     <row r="12">
@@ -849,35 +849,35 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>慢下来</t>
+          <t>事后清晨001</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>130572370</v>
+        <v>136247069</v>
       </c>
       <c r="D12" t="n">
         <v>31.08</v>
       </c>
       <c r="E12" t="n">
-        <v>1366</v>
+        <v>1414</v>
       </c>
       <c r="F12" t="n">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="G12" t="n">
-        <v>1255</v>
+        <v>1141</v>
       </c>
       <c r="H12" t="n">
-        <v>1006</v>
+        <v>1024</v>
       </c>
       <c r="I12" t="n">
-        <v>974</v>
+        <v>750</v>
       </c>
       <c r="J12" t="n">
-        <v>969</v>
+        <v>945</v>
       </c>
       <c r="K12" t="n">
-        <v>6703</v>
+        <v>6391</v>
       </c>
     </row>
     <row r="13">
@@ -886,14 +886,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>离经易道</t>
+          <t>天天中宝箱的美人</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>125755807</v>
+        <v>118016756</v>
+      </c>
+      <c r="D13" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1159</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1052</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1109</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1002</v>
+      </c>
+      <c r="I13" t="n">
+        <v>922</v>
+      </c>
+      <c r="J13" t="n">
+        <v>837</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>6081</v>
       </c>
     </row>
     <row r="14">
@@ -902,35 +923,35 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>阿騒讲没字</t>
+          <t>大鹅的后遗症</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>125618805</v>
+        <v>117882271</v>
       </c>
       <c r="D14" t="n">
         <v>31.08</v>
       </c>
       <c r="E14" t="n">
-        <v>1202.95</v>
+        <v>1218.6</v>
       </c>
       <c r="F14" t="n">
-        <v>1024.04</v>
+        <v>1069.99</v>
       </c>
       <c r="G14" t="n">
-        <v>1057.03</v>
+        <v>1017.08</v>
       </c>
       <c r="H14" t="n">
-        <v>956.21</v>
+        <v>962.6900000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>883.04</v>
+        <v>918.8</v>
       </c>
       <c r="J14" t="n">
-        <v>864.5700000000001</v>
+        <v>865.63</v>
       </c>
       <c r="K14" t="n">
-        <v>5988</v>
+        <v>6053</v>
       </c>
     </row>
     <row r="15">
@@ -939,35 +960,35 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>深深啊</t>
+          <t>阿騒讲没字</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>123832541</v>
+        <v>125618805</v>
       </c>
       <c r="D15" t="n">
         <v>31.08</v>
       </c>
       <c r="E15" t="n">
-        <v>1316.22</v>
+        <v>1202.95</v>
       </c>
       <c r="F15" t="n">
-        <v>1069.23</v>
+        <v>1024.04</v>
       </c>
       <c r="G15" t="n">
-        <v>977.39</v>
+        <v>1057.03</v>
       </c>
       <c r="H15" t="n">
-        <v>997.26</v>
+        <v>956.21</v>
       </c>
       <c r="I15" t="n">
-        <v>872.83</v>
+        <v>883.04</v>
       </c>
       <c r="J15" t="n">
-        <v>686.6799999999999</v>
+        <v>864.5700000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>5920</v>
+        <v>5988</v>
       </c>
     </row>
     <row r="16">
@@ -976,35 +997,35 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>铜锣丘</t>
+          <t>大吉大利</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>122134954</v>
+        <v>113132051</v>
       </c>
       <c r="D16" t="n">
         <v>31.08</v>
       </c>
       <c r="E16" t="n">
-        <v>1292</v>
+        <v>1246</v>
       </c>
       <c r="F16" t="n">
-        <v>984</v>
+        <v>1066</v>
       </c>
       <c r="G16" t="n">
-        <v>1027</v>
+        <v>974</v>
       </c>
       <c r="H16" t="n">
-        <v>866</v>
+        <v>928</v>
       </c>
       <c r="I16" t="n">
-        <v>895</v>
+        <v>857</v>
       </c>
       <c r="J16" t="n">
-        <v>825</v>
+        <v>903</v>
       </c>
       <c r="K16" t="n">
-        <v>5889</v>
+        <v>5974</v>
       </c>
     </row>
     <row r="17">
@@ -1013,14 +1034,35 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>一李达康一</t>
+          <t>深深啊</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>122059844</v>
+        <v>123832541</v>
+      </c>
+      <c r="D17" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1316.22</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1069.23</v>
+      </c>
+      <c r="G17" t="n">
+        <v>977.39</v>
+      </c>
+      <c r="H17" t="n">
+        <v>997.26</v>
+      </c>
+      <c r="I17" t="n">
+        <v>872.83</v>
+      </c>
+      <c r="J17" t="n">
+        <v>686.6799999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>5920</v>
       </c>
     </row>
     <row r="18">
@@ -1029,14 +1071,35 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>莫桑比克</t>
+          <t>午夜风</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>118826076</v>
+        <v>116556415</v>
+      </c>
+      <c r="D18" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1177.5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1006.3</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1079.8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>905.9</v>
+      </c>
+      <c r="I18" t="n">
+        <v>849.7</v>
+      </c>
+      <c r="J18" t="n">
+        <v>879.1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>5898</v>
       </c>
     </row>
     <row r="19">
@@ -1045,14 +1108,35 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>洋芋折耳根</t>
+          <t>铜锣丘</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>118297055</v>
+        <v>122134954</v>
+      </c>
+      <c r="D19" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1292</v>
+      </c>
+      <c r="F19" t="n">
+        <v>984</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1027</v>
+      </c>
+      <c r="H19" t="n">
+        <v>866</v>
+      </c>
+      <c r="I19" t="n">
+        <v>895</v>
+      </c>
+      <c r="J19" t="n">
+        <v>825</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>5889</v>
       </c>
     </row>
     <row r="20">
@@ -1061,35 +1145,35 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>急急如律令</t>
+          <t>离经易道</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>118746420</v>
+        <v>125755807</v>
       </c>
       <c r="D20" t="n">
-        <v>29.93</v>
+        <v>31.08</v>
       </c>
       <c r="E20" t="n">
-        <v>1220.91</v>
+        <v>1214</v>
       </c>
       <c r="F20" t="n">
-        <v>988.21</v>
+        <v>1032</v>
       </c>
       <c r="G20" t="n">
-        <v>1033.15</v>
+        <v>1030</v>
       </c>
       <c r="H20" t="n">
-        <v>999.86</v>
+        <v>927</v>
       </c>
       <c r="I20" t="n">
-        <v>859.89</v>
+        <v>901</v>
       </c>
       <c r="J20" t="n">
-        <v>693.38</v>
+        <v>738</v>
       </c>
       <c r="K20" t="n">
-        <v>5795</v>
+        <v>5842</v>
       </c>
     </row>
     <row r="21">
@@ -1098,35 +1182,35 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>天天中宝箱的美人</t>
+          <t>急急如律令</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>118016756</v>
+        <v>118746420</v>
       </c>
       <c r="D21" t="n">
         <v>31.08</v>
       </c>
       <c r="E21" t="n">
-        <v>1159</v>
+        <v>1222.91</v>
       </c>
       <c r="F21" t="n">
-        <v>1046</v>
+        <v>991.21</v>
       </c>
       <c r="G21" t="n">
-        <v>1109</v>
+        <v>1033.15</v>
       </c>
       <c r="H21" t="n">
-        <v>986</v>
+        <v>1002.86</v>
       </c>
       <c r="I21" t="n">
-        <v>909</v>
+        <v>862.89</v>
       </c>
       <c r="J21" t="n">
-        <v>825</v>
+        <v>693.38</v>
       </c>
       <c r="K21" t="n">
-        <v>6034</v>
+        <v>5806</v>
       </c>
     </row>
     <row r="22">
@@ -1135,14 +1219,35 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>听雨眠</t>
+          <t>财神爸爸</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>117992119</v>
+        <v>113588490</v>
+      </c>
+      <c r="D22" t="n">
+        <v>30.86</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1155</v>
+      </c>
+      <c r="F22" t="n">
+        <v>986</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1169</v>
+      </c>
+      <c r="H22" t="n">
+        <v>890</v>
+      </c>
+      <c r="I22" t="n">
+        <v>821</v>
+      </c>
+      <c r="J22" t="n">
+        <v>778</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>5799</v>
       </c>
     </row>
     <row r="23">
@@ -1151,35 +1256,35 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>三千道门</t>
+          <t>大丶玩家</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>117893442</v>
+        <v>116425641</v>
       </c>
       <c r="D23" t="n">
         <v>31.08</v>
       </c>
       <c r="E23" t="n">
-        <v>1075</v>
+        <v>1273</v>
       </c>
       <c r="F23" t="n">
-        <v>989.8</v>
+        <v>1017</v>
       </c>
       <c r="G23" t="n">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="H23" t="n">
-        <v>872</v>
+        <v>943</v>
       </c>
       <c r="I23" t="n">
-        <v>901</v>
+        <v>830</v>
       </c>
       <c r="J23" t="n">
-        <v>813</v>
+        <v>687</v>
       </c>
       <c r="K23" t="n">
-        <v>5690</v>
+        <v>5791</v>
       </c>
     </row>
     <row r="24">
@@ -1188,14 +1293,35 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>大鹅的后遗症</t>
+          <t>大鹅的小号</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>117882271</v>
+        <v>111588664</v>
+      </c>
+      <c r="D24" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1184.03</v>
+      </c>
+      <c r="F24" t="n">
+        <v>992.86</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1061.8</v>
+      </c>
+      <c r="H24" t="n">
+        <v>919.89</v>
+      </c>
+      <c r="I24" t="n">
+        <v>844.3200000000001</v>
+      </c>
+      <c r="J24" t="n">
+        <v>785.21</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>5788</v>
       </c>
     </row>
     <row r="25">
@@ -1204,35 +1330,35 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>午夜风</t>
+          <t>污妖王</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>116556415</v>
+        <v>109569104</v>
       </c>
       <c r="D25" t="n">
         <v>31.08</v>
       </c>
       <c r="E25" t="n">
-        <v>1177.5</v>
+        <v>1206.22</v>
       </c>
       <c r="F25" t="n">
-        <v>1006.3</v>
+        <v>973.33</v>
       </c>
       <c r="G25" t="n">
-        <v>1079.8</v>
+        <v>1108.64</v>
       </c>
       <c r="H25" t="n">
-        <v>905.9</v>
+        <v>927.3099999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>849.7</v>
+        <v>839.75</v>
       </c>
       <c r="J25" t="n">
-        <v>879.1</v>
+        <v>715.5599999999999</v>
       </c>
       <c r="K25" t="n">
-        <v>5898</v>
+        <v>5771</v>
       </c>
     </row>
     <row r="26">
@@ -1241,14 +1367,35 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>大丶玩家</t>
+          <t>流寇头目</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>116425641</v>
+        <v>115849112</v>
+      </c>
+      <c r="D26" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1262.62</v>
+      </c>
+      <c r="F26" t="n">
+        <v>993.62</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1019.13</v>
+      </c>
+      <c r="H26" t="n">
+        <v>863</v>
+      </c>
+      <c r="I26" t="n">
+        <v>878.74</v>
+      </c>
+      <c r="J26" t="n">
+        <v>722.2</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>5739</v>
       </c>
     </row>
     <row r="27">
@@ -1257,14 +1404,35 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>锦衣卫金蝉子</t>
+          <t>我佛了</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>116188284</v>
+        <v>114015965</v>
+      </c>
+      <c r="D27" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1042.35</v>
+      </c>
+      <c r="F27" t="n">
+        <v>989.6799999999999</v>
+      </c>
+      <c r="G27" t="n">
+        <v>992.66</v>
+      </c>
+      <c r="H27" t="n">
+        <v>931.78</v>
+      </c>
+      <c r="I27" t="n">
+        <v>882.66</v>
+      </c>
+      <c r="J27" t="n">
+        <v>872.66</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>5712</v>
       </c>
     </row>
     <row r="28">
@@ -1273,35 +1441,35 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>流寇头目</t>
+          <t>三千道门</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>115849112</v>
+        <v>117893442</v>
       </c>
       <c r="D28" t="n">
         <v>31.08</v>
       </c>
       <c r="E28" t="n">
-        <v>1262.62</v>
+        <v>1075</v>
       </c>
       <c r="F28" t="n">
-        <v>993.62</v>
+        <v>989.8</v>
       </c>
       <c r="G28" t="n">
-        <v>1019.13</v>
+        <v>1039</v>
       </c>
       <c r="H28" t="n">
-        <v>863</v>
+        <v>872</v>
       </c>
       <c r="I28" t="n">
-        <v>878.74</v>
+        <v>901</v>
       </c>
       <c r="J28" t="n">
-        <v>722.2</v>
+        <v>813</v>
       </c>
       <c r="K28" t="n">
-        <v>5739</v>
+        <v>5690</v>
       </c>
     </row>
     <row r="29">
@@ -1316,8 +1484,29 @@
       <c r="C29" t="n">
         <v>114900115</v>
       </c>
+      <c r="D29" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1188.25</v>
+      </c>
+      <c r="F29" t="n">
+        <v>890.33</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1010.39</v>
+      </c>
+      <c r="H29" t="n">
+        <v>853.4400000000001</v>
+      </c>
+      <c r="I29" t="n">
+        <v>920.21</v>
+      </c>
+      <c r="J29" t="n">
+        <v>824.8</v>
+      </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>5687</v>
       </c>
     </row>
     <row r="30">
@@ -1326,35 +1515,35 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>财神爸爸</t>
+          <t>荒天帝</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>113588490</v>
+        <v>106280718</v>
       </c>
       <c r="D30" t="n">
-        <v>30.86</v>
+        <v>30.48</v>
       </c>
       <c r="E30" t="n">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="F30" t="n">
-        <v>986</v>
+        <v>939</v>
       </c>
       <c r="G30" t="n">
-        <v>1169</v>
+        <v>950</v>
       </c>
       <c r="H30" t="n">
-        <v>890</v>
+        <v>880</v>
       </c>
       <c r="I30" t="n">
-        <v>821</v>
+        <v>857</v>
       </c>
       <c r="J30" t="n">
-        <v>778</v>
+        <v>876</v>
       </c>
       <c r="K30" t="n">
-        <v>5799</v>
+        <v>5656</v>
       </c>
     </row>
     <row r="31">
@@ -1363,35 +1552,35 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>我佛了</t>
+          <t>太可怜了丶</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>114015965</v>
+        <v>112811033</v>
       </c>
       <c r="D31" t="n">
         <v>31.08</v>
       </c>
       <c r="E31" t="n">
-        <v>1042.35</v>
+        <v>1131.99</v>
       </c>
       <c r="F31" t="n">
-        <v>989.6799999999999</v>
+        <v>945.03</v>
       </c>
       <c r="G31" t="n">
-        <v>992.66</v>
+        <v>1038.24</v>
       </c>
       <c r="H31" t="n">
-        <v>931.78</v>
+        <v>795.75</v>
       </c>
       <c r="I31" t="n">
-        <v>882.66</v>
+        <v>856.86</v>
       </c>
       <c r="J31" t="n">
-        <v>872.66</v>
+        <v>850.35</v>
       </c>
       <c r="K31" t="n">
-        <v>5712</v>
+        <v>5618</v>
       </c>
     </row>
     <row r="32">
@@ -1400,35 +1589,35 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>露芜衣小狐狸</t>
+          <t>喳喳喳</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>113525199</v>
+        <v>111598239</v>
       </c>
       <c r="D32" t="n">
-        <v>31.08</v>
+        <v>29.27</v>
       </c>
       <c r="E32" t="n">
-        <v>1167</v>
+        <v>1196.65</v>
       </c>
       <c r="F32" t="n">
-        <v>980</v>
+        <v>954.59</v>
       </c>
       <c r="G32" t="n">
-        <v>985</v>
+        <v>1038.99</v>
       </c>
       <c r="H32" t="n">
-        <v>915</v>
+        <v>857.27</v>
       </c>
       <c r="I32" t="n">
-        <v>829</v>
+        <v>820.77</v>
       </c>
       <c r="J32" t="n">
-        <v>715</v>
+        <v>749.23</v>
       </c>
       <c r="K32" t="n">
-        <v>5591</v>
+        <v>5618</v>
       </c>
     </row>
     <row r="33">
@@ -1437,35 +1626,35 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>大吉大利</t>
+          <t>露芜衣小狐狸</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>113132051</v>
+        <v>113525199</v>
       </c>
       <c r="D33" t="n">
         <v>31.08</v>
       </c>
       <c r="E33" t="n">
-        <v>1246</v>
+        <v>1167</v>
       </c>
       <c r="F33" t="n">
-        <v>1066</v>
+        <v>980</v>
       </c>
       <c r="G33" t="n">
-        <v>974</v>
+        <v>985</v>
       </c>
       <c r="H33" t="n">
-        <v>928</v>
+        <v>915</v>
       </c>
       <c r="I33" t="n">
-        <v>857</v>
+        <v>829</v>
       </c>
       <c r="J33" t="n">
-        <v>903</v>
+        <v>715</v>
       </c>
       <c r="K33" t="n">
-        <v>5974</v>
+        <v>5591</v>
       </c>
     </row>
     <row r="34">
@@ -1474,35 +1663,35 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>太可怜了丶</t>
+          <t>随遇而安#732</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>112811033</v>
+        <v>109120971</v>
       </c>
       <c r="D34" t="n">
-        <v>31.08</v>
+        <v>30.48</v>
       </c>
       <c r="E34" t="n">
-        <v>1131.99</v>
+        <v>1113</v>
       </c>
       <c r="F34" t="n">
-        <v>945.03</v>
+        <v>942</v>
       </c>
       <c r="G34" t="n">
-        <v>1038.24</v>
+        <v>1023</v>
       </c>
       <c r="H34" t="n">
-        <v>795.75</v>
+        <v>959</v>
       </c>
       <c r="I34" t="n">
-        <v>856.86</v>
+        <v>836</v>
       </c>
       <c r="J34" t="n">
-        <v>850.35</v>
+        <v>714</v>
       </c>
       <c r="K34" t="n">
-        <v>5618</v>
+        <v>5587</v>
       </c>
     </row>
     <row r="35">
@@ -1511,14 +1700,35 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>零壹贰壹</t>
+          <t>三宅一生</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>111853555</v>
+        <v>111581031</v>
+      </c>
+      <c r="D35" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1190.51</v>
+      </c>
+      <c r="F35" t="n">
+        <v>960.49</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1003.69</v>
+      </c>
+      <c r="H35" t="n">
+        <v>874</v>
+      </c>
+      <c r="I35" t="n">
+        <v>809.75</v>
+      </c>
+      <c r="J35" t="n">
+        <v>742.05</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>5580</v>
       </c>
     </row>
     <row r="36">
@@ -1527,14 +1737,35 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>喳喳喳</t>
+          <t>浮萍之末</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>111598239</v>
+        <v>109678977</v>
+      </c>
+      <c r="D36" t="n">
+        <v>30</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1103</v>
+      </c>
+      <c r="F36" t="n">
+        <v>955</v>
+      </c>
+      <c r="G36" t="n">
+        <v>945</v>
+      </c>
+      <c r="H36" t="n">
+        <v>840</v>
+      </c>
+      <c r="I36" t="n">
+        <v>854</v>
+      </c>
+      <c r="J36" t="n">
+        <v>848</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>5545</v>
       </c>
     </row>
     <row r="37">
@@ -1543,35 +1774,35 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>大鹅的小号</t>
+          <t>早日武统</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>111588664</v>
+        <v>109640870</v>
       </c>
       <c r="D37" t="n">
         <v>31.08</v>
       </c>
       <c r="E37" t="n">
-        <v>1184.03</v>
+        <v>1054</v>
       </c>
       <c r="F37" t="n">
-        <v>992.86</v>
+        <v>923</v>
       </c>
       <c r="G37" t="n">
-        <v>1061.8</v>
+        <v>980</v>
       </c>
       <c r="H37" t="n">
-        <v>919.89</v>
+        <v>919</v>
       </c>
       <c r="I37" t="n">
-        <v>844.3200000000001</v>
+        <v>836</v>
       </c>
       <c r="J37" t="n">
-        <v>785.21</v>
+        <v>750</v>
       </c>
       <c r="K37" t="n">
-        <v>5788</v>
+        <v>5462</v>
       </c>
     </row>
     <row r="38">
@@ -1580,35 +1811,35 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>三宅一生</t>
+          <t>鱼老六</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>111581031</v>
+        <v>102990422</v>
       </c>
       <c r="D38" t="n">
-        <v>31.08</v>
+        <v>30.32</v>
       </c>
       <c r="E38" t="n">
-        <v>1190.51</v>
+        <v>1053.33</v>
       </c>
       <c r="F38" t="n">
-        <v>960.49</v>
+        <v>929.6900000000001</v>
       </c>
       <c r="G38" t="n">
-        <v>1003.69</v>
+        <v>969.5599999999999</v>
       </c>
       <c r="H38" t="n">
-        <v>874</v>
+        <v>838.71</v>
       </c>
       <c r="I38" t="n">
-        <v>809.75</v>
+        <v>788.79</v>
       </c>
       <c r="J38" t="n">
-        <v>742.05</v>
+        <v>825.67</v>
       </c>
       <c r="K38" t="n">
-        <v>5580</v>
+        <v>5406</v>
       </c>
     </row>
     <row r="39">
@@ -1617,35 +1848,35 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>月下星河涟漪</t>
+          <t>换啥名呢</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>110502257</v>
+        <v>110242916</v>
       </c>
       <c r="D39" t="n">
-        <v>30.32</v>
+        <v>31.08</v>
       </c>
       <c r="E39" t="n">
-        <v>1101.1</v>
+        <v>981.89</v>
       </c>
       <c r="F39" t="n">
-        <v>867.63</v>
+        <v>958.92</v>
       </c>
       <c r="G39" t="n">
-        <v>879.36</v>
+        <v>935.11</v>
       </c>
       <c r="H39" t="n">
-        <v>811.35</v>
+        <v>904.65</v>
       </c>
       <c r="I39" t="n">
-        <v>829.91</v>
+        <v>848.8</v>
       </c>
       <c r="J39" t="n">
-        <v>778.8200000000001</v>
+        <v>760.0599999999999</v>
       </c>
       <c r="K39" t="n">
-        <v>5268</v>
+        <v>5389</v>
       </c>
     </row>
     <row r="40">
@@ -1654,14 +1885,35 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>换啥名呢</t>
+          <t>冰凉灬丶</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>110242916</v>
+        <v>109784982</v>
+      </c>
+      <c r="D40" t="n">
+        <v>29.28</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1056.03</v>
+      </c>
+      <c r="F40" t="n">
+        <v>916.96</v>
+      </c>
+      <c r="G40" t="n">
+        <v>940.77</v>
+      </c>
+      <c r="H40" t="n">
+        <v>830.7</v>
+      </c>
+      <c r="I40" t="n">
+        <v>865.05</v>
+      </c>
+      <c r="J40" t="n">
+        <v>757.64</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>5367</v>
       </c>
     </row>
     <row r="41">
@@ -1670,14 +1922,35 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>一匹天涯的马</t>
+          <t>沉睡伊人</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>110108327</v>
+        <v>104679115</v>
+      </c>
+      <c r="D41" t="n">
+        <v>29.28</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1043.72</v>
+      </c>
+      <c r="F41" t="n">
+        <v>942.59</v>
+      </c>
+      <c r="G41" t="n">
+        <v>959.42</v>
+      </c>
+      <c r="H41" t="n">
+        <v>905.4299999999999</v>
+      </c>
+      <c r="I41" t="n">
+        <v>855.88</v>
+      </c>
+      <c r="J41" t="n">
+        <v>595.21</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>5302</v>
       </c>
     </row>
     <row r="42">
@@ -1686,14 +1959,35 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>传龙天下</t>
+          <t>月下星河涟漪</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>109978751</v>
+        <v>110502257</v>
+      </c>
+      <c r="D42" t="n">
+        <v>30.32</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1101.1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>867.63</v>
+      </c>
+      <c r="G42" t="n">
+        <v>879.36</v>
+      </c>
+      <c r="H42" t="n">
+        <v>811.35</v>
+      </c>
+      <c r="I42" t="n">
+        <v>829.91</v>
+      </c>
+      <c r="J42" t="n">
+        <v>778.8200000000001</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>5268</v>
       </c>
     </row>
     <row r="43">
@@ -1702,35 +1996,35 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>冰凉灬丶</t>
+          <t>又见春</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>109784982</v>
+        <v>100654578</v>
       </c>
       <c r="D43" t="n">
-        <v>29.28</v>
+        <v>31.08</v>
       </c>
       <c r="E43" t="n">
-        <v>1056.03</v>
+        <v>1083.88</v>
       </c>
       <c r="F43" t="n">
-        <v>916.96</v>
+        <v>924.3</v>
       </c>
       <c r="G43" t="n">
-        <v>940.77</v>
+        <v>928.17</v>
       </c>
       <c r="H43" t="n">
-        <v>830.7</v>
+        <v>887.6799999999999</v>
       </c>
       <c r="I43" t="n">
-        <v>865.05</v>
+        <v>882.3</v>
       </c>
       <c r="J43" t="n">
-        <v>757.64</v>
+        <v>561.1799999999999</v>
       </c>
       <c r="K43" t="n">
-        <v>5367</v>
+        <v>5268</v>
       </c>
     </row>
     <row r="44">
@@ -1739,14 +2033,35 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>红太狼</t>
+          <t>小草马</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>109732694</v>
+        <v>102575977</v>
+      </c>
+      <c r="D44" t="n">
+        <v>30.04</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1014.98</v>
+      </c>
+      <c r="F44" t="n">
+        <v>890.83</v>
+      </c>
+      <c r="G44" t="n">
+        <v>868.86</v>
+      </c>
+      <c r="H44" t="n">
+        <v>891.6</v>
+      </c>
+      <c r="I44" t="n">
+        <v>827.67</v>
+      </c>
+      <c r="J44" t="n">
+        <v>760.4299999999999</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>5254</v>
       </c>
     </row>
     <row r="45">
@@ -1755,35 +2070,35 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>浮萍之末</t>
+          <t>是阿饼</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>109678977</v>
+        <v>108930820</v>
       </c>
       <c r="D45" t="n">
-        <v>30</v>
+        <v>30.48</v>
       </c>
       <c r="E45" t="n">
-        <v>1103</v>
+        <v>1063</v>
       </c>
       <c r="F45" t="n">
-        <v>955</v>
+        <v>934</v>
       </c>
       <c r="G45" t="n">
-        <v>945</v>
+        <v>901</v>
       </c>
       <c r="H45" t="n">
-        <v>840</v>
+        <v>873</v>
       </c>
       <c r="I45" t="n">
-        <v>854</v>
+        <v>834</v>
       </c>
       <c r="J45" t="n">
-        <v>848</v>
+        <v>637</v>
       </c>
       <c r="K45" t="n">
-        <v>5545</v>
+        <v>5242</v>
       </c>
     </row>
     <row r="46">
@@ -1792,14 +2107,35 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>早日武统</t>
+          <t>凡尘琐事多</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>109640870</v>
+        <v>105229464</v>
+      </c>
+      <c r="D46" t="n">
+        <v>28.52</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1108.09</v>
+      </c>
+      <c r="F46" t="n">
+        <v>937.45</v>
+      </c>
+      <c r="G46" t="n">
+        <v>868.62</v>
+      </c>
+      <c r="H46" t="n">
+        <v>929.77</v>
+      </c>
+      <c r="I46" t="n">
+        <v>763.4400000000001</v>
+      </c>
+      <c r="J46" t="n">
+        <v>613.8</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>5221</v>
       </c>
     </row>
     <row r="47">
@@ -1808,14 +2144,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>秋刀齐爽</t>
+          <t>清热化毒丸</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>109628070</v>
+        <v>104153322</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1085</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1002</v>
+      </c>
+      <c r="G47" t="n">
+        <v>840</v>
+      </c>
+      <c r="H47" t="n">
+        <v>860</v>
+      </c>
+      <c r="I47" t="n">
+        <v>761</v>
+      </c>
+      <c r="J47" t="n">
+        <v>640</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>5188</v>
       </c>
     </row>
     <row r="48">
@@ -1824,35 +2178,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>污妖王</t>
+          <t>凤凰城</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>109569104</v>
-      </c>
-      <c r="D48" t="n">
-        <v>31.08</v>
+        <v>104997066</v>
       </c>
       <c r="E48" t="n">
-        <v>1206.22</v>
+        <v>1028.89</v>
       </c>
       <c r="F48" t="n">
-        <v>973.33</v>
+        <v>848.34</v>
       </c>
       <c r="G48" t="n">
-        <v>1108.64</v>
+        <v>958.0599999999999</v>
       </c>
       <c r="H48" t="n">
-        <v>927.3099999999999</v>
+        <v>860.67</v>
       </c>
       <c r="I48" t="n">
-        <v>839.75</v>
+        <v>825.6799999999999</v>
       </c>
       <c r="J48" t="n">
-        <v>715.5599999999999</v>
+        <v>632.85</v>
       </c>
       <c r="K48" t="n">
-        <v>5771</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="49">
@@ -1861,14 +2212,35 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>哈特虎</t>
+          <t>布小丁</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>109254507</v>
+        <v>100116626</v>
+      </c>
+      <c r="D49" t="n">
+        <v>30.15</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1017.75</v>
+      </c>
+      <c r="F49" t="n">
+        <v>894.52</v>
+      </c>
+      <c r="G49" t="n">
+        <v>830.88</v>
+      </c>
+      <c r="H49" t="n">
+        <v>857.28</v>
+      </c>
+      <c r="I49" t="n">
+        <v>854.9299999999999</v>
+      </c>
+      <c r="J49" t="n">
+        <v>670.52</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>5126</v>
       </c>
     </row>
     <row r="50">
@@ -1877,35 +2249,35 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>随遇而安#732</t>
+          <t>哈特虎</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>109120971</v>
+        <v>109254507</v>
       </c>
       <c r="D50" t="n">
-        <v>30.48</v>
+        <v>29.56</v>
       </c>
       <c r="E50" t="n">
-        <v>1113</v>
+        <v>850.09</v>
       </c>
       <c r="F50" t="n">
-        <v>942</v>
+        <v>882.5</v>
       </c>
       <c r="G50" t="n">
-        <v>1023</v>
+        <v>911.0700000000001</v>
       </c>
       <c r="H50" t="n">
-        <v>959</v>
+        <v>899.09</v>
       </c>
       <c r="I50" t="n">
-        <v>836</v>
+        <v>800.2</v>
       </c>
       <c r="J50" t="n">
-        <v>714</v>
+        <v>663.86</v>
       </c>
       <c r="K50" t="n">
-        <v>5587</v>
+        <v>5007</v>
       </c>
     </row>
     <row r="51">
@@ -1914,14 +2286,35 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>是阿饼</t>
+          <t>红太狼</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>108930820</v>
+        <v>109732694</v>
+      </c>
+      <c r="D51" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E51" t="n">
+        <v>900</v>
+      </c>
+      <c r="F51" t="n">
+        <v>900</v>
+      </c>
+      <c r="G51" t="n">
+        <v>800</v>
+      </c>
+      <c r="H51" t="n">
+        <v>800</v>
+      </c>
+      <c r="I51" t="n">
+        <v>800</v>
+      </c>
+      <c r="J51" t="n">
+        <v>800</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="52">
@@ -1930,14 +2323,35 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>月泠瑶</t>
+          <t>貂蝉是白嫖的神</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>108840139</v>
+        <v>102903505</v>
+      </c>
+      <c r="D52" t="n">
+        <v>30.32</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1069.51</v>
+      </c>
+      <c r="F52" t="n">
+        <v>826.96</v>
+      </c>
+      <c r="G52" t="n">
+        <v>752.63</v>
+      </c>
+      <c r="H52" t="n">
+        <v>827.55</v>
+      </c>
+      <c r="I52" t="n">
+        <v>725.5599999999999</v>
+      </c>
+      <c r="J52" t="n">
+        <v>785.89</v>
       </c>
       <c r="K52" t="n">
-        <v>0</v>
+        <v>4988</v>
       </c>
     </row>
     <row r="53">
@@ -1946,14 +2360,35 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>消失的眼袋</t>
+          <t>叶孤城</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>108094113</v>
+        <v>106652395</v>
+      </c>
+      <c r="D53" t="n">
+        <v>30.75</v>
+      </c>
+      <c r="E53" t="n">
+        <v>992.48</v>
+      </c>
+      <c r="F53" t="n">
+        <v>886.13</v>
+      </c>
+      <c r="G53" t="n">
+        <v>773.78</v>
+      </c>
+      <c r="H53" t="n">
+        <v>805.22</v>
+      </c>
+      <c r="I53" t="n">
+        <v>816.71</v>
+      </c>
+      <c r="J53" t="n">
+        <v>700.8</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>4975</v>
       </c>
     </row>
     <row r="54">
@@ -1962,14 +2397,35 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>看星星</t>
+          <t>厉害的桃夭</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>108027627</v>
+        <v>91058618</v>
+      </c>
+      <c r="D54" t="n">
+        <v>29.72</v>
+      </c>
+      <c r="E54" t="n">
+        <v>883.04</v>
+      </c>
+      <c r="F54" t="n">
+        <v>841.23</v>
+      </c>
+      <c r="G54" t="n">
+        <v>848.01</v>
+      </c>
+      <c r="H54" t="n">
+        <v>896.9</v>
+      </c>
+      <c r="I54" t="n">
+        <v>779.01</v>
+      </c>
+      <c r="J54" t="n">
+        <v>723.8099999999999</v>
       </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>4972</v>
       </c>
     </row>
     <row r="55">
@@ -1984,8 +2440,29 @@
       <c r="C55" t="n">
         <v>107231360</v>
       </c>
+      <c r="D55" t="n">
+        <v>29.23</v>
+      </c>
+      <c r="E55" t="n">
+        <v>964.05</v>
+      </c>
+      <c r="F55" t="n">
+        <v>902.49</v>
+      </c>
+      <c r="G55" t="n">
+        <v>773.02</v>
+      </c>
+      <c r="H55" t="n">
+        <v>809.49</v>
+      </c>
+      <c r="I55" t="n">
+        <v>809.1900000000001</v>
+      </c>
+      <c r="J55" t="n">
+        <v>669.08</v>
+      </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>4927</v>
       </c>
     </row>
     <row r="56">
@@ -1994,35 +2471,35 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>叶孤城</t>
+          <t>爱吃羊肉</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>106652395</v>
+        <v>97473105</v>
       </c>
       <c r="D56" t="n">
-        <v>30.75</v>
+        <v>29.72</v>
       </c>
       <c r="E56" t="n">
-        <v>992.48</v>
+        <v>857</v>
       </c>
       <c r="F56" t="n">
-        <v>886.13</v>
+        <v>840</v>
       </c>
       <c r="G56" t="n">
-        <v>773.78</v>
+        <v>818</v>
       </c>
       <c r="H56" t="n">
-        <v>805.22</v>
+        <v>789</v>
       </c>
       <c r="I56" t="n">
-        <v>816.71</v>
+        <v>800</v>
       </c>
       <c r="J56" t="n">
-        <v>700.8</v>
+        <v>792</v>
       </c>
       <c r="K56" t="n">
-        <v>4975</v>
+        <v>4896</v>
       </c>
     </row>
     <row r="57">
@@ -2031,35 +2508,35 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>荒天帝</t>
+          <t>叶落落</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>106280718</v>
+        <v>97976695</v>
       </c>
       <c r="D57" t="n">
-        <v>30.48</v>
+        <v>29.01</v>
       </c>
       <c r="E57" t="n">
-        <v>1154</v>
+        <v>928.1</v>
       </c>
       <c r="F57" t="n">
-        <v>939</v>
+        <v>876.51</v>
       </c>
       <c r="G57" t="n">
-        <v>950</v>
+        <v>765.6900000000001</v>
       </c>
       <c r="H57" t="n">
-        <v>880</v>
+        <v>790.29</v>
       </c>
       <c r="I57" t="n">
-        <v>857</v>
+        <v>817.84</v>
       </c>
       <c r="J57" t="n">
-        <v>876</v>
+        <v>681.3099999999999</v>
       </c>
       <c r="K57" t="n">
-        <v>5656</v>
+        <v>4860</v>
       </c>
     </row>
     <row r="58">
@@ -2068,35 +2545,35 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>神乎其技的男人</t>
+          <t>寳尐姐</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>105730651</v>
+        <v>90692097</v>
       </c>
       <c r="D58" t="n">
-        <v>29.56</v>
+        <v>29.72</v>
       </c>
       <c r="E58" t="n">
-        <v>840.9</v>
+        <v>950.7</v>
       </c>
       <c r="F58" t="n">
-        <v>887.71</v>
+        <v>778.28</v>
       </c>
       <c r="G58" t="n">
-        <v>664.59</v>
+        <v>764.645</v>
       </c>
       <c r="H58" t="n">
-        <v>788.8</v>
+        <v>760.28</v>
       </c>
       <c r="I58" t="n">
-        <v>740.3</v>
+        <v>752.12</v>
       </c>
       <c r="J58" t="n">
-        <v>584.62</v>
+        <v>749.7</v>
       </c>
       <c r="K58" t="n">
-        <v>4507</v>
+        <v>4756</v>
       </c>
     </row>
     <row r="59">
@@ -2105,14 +2582,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>玄门丶麟墨</t>
+          <t>和事佬</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>105527080</v>
+        <v>100391957</v>
+      </c>
+      <c r="E59" t="n">
+        <v>808</v>
+      </c>
+      <c r="F59" t="n">
+        <v>879</v>
+      </c>
+      <c r="G59" t="n">
+        <v>796</v>
+      </c>
+      <c r="H59" t="n">
+        <v>810</v>
+      </c>
+      <c r="I59" t="n">
+        <v>775</v>
+      </c>
+      <c r="J59" t="n">
+        <v>666</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>4734</v>
       </c>
     </row>
     <row r="60">
@@ -2121,14 +2616,35 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>凡尘琐事多</t>
+          <t>爱吃肉的棒同学</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>105229464</v>
+        <v>96025973</v>
+      </c>
+      <c r="D60" t="n">
+        <v>29.06</v>
+      </c>
+      <c r="E60" t="n">
+        <v>907.36</v>
+      </c>
+      <c r="F60" t="n">
+        <v>884.8200000000001</v>
+      </c>
+      <c r="G60" t="n">
+        <v>768.45</v>
+      </c>
+      <c r="H60" t="n">
+        <v>792.75</v>
+      </c>
+      <c r="I60" t="n">
+        <v>736.53</v>
+      </c>
+      <c r="J60" t="n">
+        <v>551.96</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>4642</v>
       </c>
     </row>
     <row r="61">
@@ -2137,14 +2653,35 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>凤凰城</t>
+          <t>扁豆焖面</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>104997066</v>
+        <v>95033759</v>
+      </c>
+      <c r="D61" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="E61" t="n">
+        <v>922.26</v>
+      </c>
+      <c r="F61" t="n">
+        <v>828.41</v>
+      </c>
+      <c r="G61" t="n">
+        <v>762.1</v>
+      </c>
+      <c r="H61" t="n">
+        <v>838.09</v>
+      </c>
+      <c r="I61" t="n">
+        <v>711.13</v>
+      </c>
+      <c r="J61" t="n">
+        <v>537.79</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="62">
@@ -2153,35 +2690,35 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>沉睡伊人</t>
+          <t>嘉嘉嘉</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>104679115</v>
+        <v>99678853</v>
       </c>
       <c r="D62" t="n">
-        <v>29.28</v>
+        <v>27.32</v>
       </c>
       <c r="E62" t="n">
-        <v>1043.72</v>
+        <v>769.88</v>
       </c>
       <c r="F62" t="n">
-        <v>942.59</v>
+        <v>846.61</v>
       </c>
       <c r="G62" t="n">
-        <v>959.42</v>
+        <v>734.58</v>
       </c>
       <c r="H62" t="n">
-        <v>905.4299999999999</v>
+        <v>849.92</v>
       </c>
       <c r="I62" t="n">
-        <v>855.88</v>
+        <v>754.0700000000001</v>
       </c>
       <c r="J62" t="n">
-        <v>595.21</v>
+        <v>644.1</v>
       </c>
       <c r="K62" t="n">
-        <v>5302</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="63">
@@ -2190,14 +2727,35 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>小怪兽</t>
+          <t>西点啊</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>104547156</v>
+        <v>96935146</v>
+      </c>
+      <c r="D63" t="n">
+        <v>26.16</v>
+      </c>
+      <c r="E63" t="n">
+        <v>801</v>
+      </c>
+      <c r="F63" t="n">
+        <v>836</v>
+      </c>
+      <c r="G63" t="n">
+        <v>867</v>
+      </c>
+      <c r="H63" t="n">
+        <v>857</v>
+      </c>
+      <c r="I63" t="n">
+        <v>677</v>
+      </c>
+      <c r="J63" t="n">
+        <v>558</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>4596</v>
       </c>
     </row>
     <row r="64">
@@ -2206,14 +2764,35 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>龙吟天下</t>
+          <t>神乎其技的男人</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>104441967</v>
+        <v>105730651</v>
+      </c>
+      <c r="D64" t="n">
+        <v>29.56</v>
+      </c>
+      <c r="E64" t="n">
+        <v>840.9</v>
+      </c>
+      <c r="F64" t="n">
+        <v>887.71</v>
+      </c>
+      <c r="G64" t="n">
+        <v>664.59</v>
+      </c>
+      <c r="H64" t="n">
+        <v>788.8</v>
+      </c>
+      <c r="I64" t="n">
+        <v>740.3</v>
+      </c>
+      <c r="J64" t="n">
+        <v>584.62</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>4507</v>
       </c>
     </row>
     <row r="65">
@@ -2222,32 +2801,35 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>清热化毒丸</t>
+          <t>啊霞霞霞</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>104153322</v>
+        <v>93773887</v>
+      </c>
+      <c r="D65" t="n">
+        <v>27</v>
       </c>
       <c r="E65" t="n">
-        <v>1085</v>
+        <v>948.78</v>
       </c>
       <c r="F65" t="n">
-        <v>1002</v>
+        <v>810.22</v>
       </c>
       <c r="G65" t="n">
-        <v>840</v>
+        <v>641.73</v>
       </c>
       <c r="H65" t="n">
-        <v>860</v>
+        <v>777.63</v>
       </c>
       <c r="I65" t="n">
-        <v>761</v>
+        <v>749.95</v>
       </c>
       <c r="J65" t="n">
-        <v>640</v>
+        <v>568.64</v>
       </c>
       <c r="K65" t="n">
-        <v>5188</v>
+        <v>4497</v>
       </c>
     </row>
     <row r="66">
@@ -2256,35 +2838,35 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>鱼老六</t>
+          <t>天天骑奉孝夫人</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>102990422</v>
+        <v>96072613</v>
       </c>
       <c r="D66" t="n">
-        <v>30.32</v>
+        <v>27.8</v>
       </c>
       <c r="E66" t="n">
-        <v>1053.33</v>
+        <v>680.3200000000001</v>
       </c>
       <c r="F66" t="n">
-        <v>929.6900000000001</v>
+        <v>877.98</v>
       </c>
       <c r="G66" t="n">
-        <v>969.5599999999999</v>
+        <v>684.0599999999999</v>
       </c>
       <c r="H66" t="n">
-        <v>838.71</v>
+        <v>810.62</v>
       </c>
       <c r="I66" t="n">
-        <v>788.79</v>
+        <v>775.24</v>
       </c>
       <c r="J66" t="n">
-        <v>825.67</v>
+        <v>546.17</v>
       </c>
       <c r="K66" t="n">
-        <v>5406</v>
+        <v>4374</v>
       </c>
     </row>
     <row r="67">
@@ -2293,35 +2875,35 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>貂蝉是白嫖的神</t>
+          <t>地产最少小号</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>102903505</v>
+        <v>91209747</v>
       </c>
       <c r="D67" t="n">
-        <v>30.32</v>
+        <v>28.96</v>
       </c>
       <c r="E67" t="n">
-        <v>1069.51</v>
+        <v>690.02</v>
       </c>
       <c r="F67" t="n">
-        <v>826.96</v>
+        <v>829.73</v>
       </c>
       <c r="G67" t="n">
-        <v>752.63</v>
+        <v>818.35</v>
       </c>
       <c r="H67" t="n">
-        <v>827.55</v>
+        <v>775.9</v>
       </c>
       <c r="I67" t="n">
-        <v>725.5599999999999</v>
+        <v>701.47</v>
       </c>
       <c r="J67" t="n">
-        <v>785.89</v>
+        <v>514.15</v>
       </c>
       <c r="K67" t="n">
-        <v>4988</v>
+        <v>4330</v>
       </c>
     </row>
     <row r="68">
@@ -2330,14 +2912,35 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>与落日道晚安</t>
+          <t>依旧安然</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>102704381</v>
+        <v>93246301</v>
+      </c>
+      <c r="D68" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="E68" t="n">
+        <v>700.84</v>
+      </c>
+      <c r="F68" t="n">
+        <v>761.8200000000001</v>
+      </c>
+      <c r="G68" t="n">
+        <v>717.38</v>
+      </c>
+      <c r="H68" t="n">
+        <v>784.0599999999999</v>
+      </c>
+      <c r="I68" t="n">
+        <v>716.74</v>
+      </c>
+      <c r="J68" t="n">
+        <v>628.74</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>4310</v>
       </c>
     </row>
     <row r="69">
@@ -2346,14 +2949,35 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>小草马</t>
+          <t>糖菓児</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>102575977</v>
+        <v>91717455</v>
+      </c>
+      <c r="D69" t="n">
+        <v>29.12</v>
+      </c>
+      <c r="E69" t="n">
+        <v>641.34</v>
+      </c>
+      <c r="F69" t="n">
+        <v>777.33</v>
+      </c>
+      <c r="G69" t="n">
+        <v>596.41</v>
+      </c>
+      <c r="H69" t="n">
+        <v>775.55</v>
+      </c>
+      <c r="I69" t="n">
+        <v>776.76</v>
+      </c>
+      <c r="J69" t="n">
+        <v>621.87</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>4189</v>
       </c>
     </row>
     <row r="70">
@@ -2362,14 +2986,35 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>小乔啊</t>
+          <t>洛洛233</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>101251332</v>
+        <v>100755796</v>
+      </c>
+      <c r="D70" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="E70" t="n">
+        <v>657.79</v>
+      </c>
+      <c r="F70" t="n">
+        <v>829.1</v>
+      </c>
+      <c r="G70" t="n">
+        <v>659.97</v>
+      </c>
+      <c r="H70" t="n">
+        <v>795.8099999999999</v>
+      </c>
+      <c r="I70" t="n">
+        <v>671.76</v>
+      </c>
+      <c r="J70" t="n">
+        <v>506.38</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>4121</v>
       </c>
     </row>
     <row r="71">
@@ -2378,14 +3023,35 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>洛洛233</t>
+          <t>小怪兽</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>100755796</v>
+        <v>104547156</v>
+      </c>
+      <c r="D71" t="n">
+        <v>29.06</v>
+      </c>
+      <c r="E71" t="n">
+        <v>899.62</v>
+      </c>
+      <c r="F71" t="n">
+        <v>858.49</v>
+      </c>
+      <c r="G71" t="n">
+        <v>716.33</v>
+      </c>
+      <c r="H71" t="n">
+        <v>790.1900000000001</v>
+      </c>
+      <c r="I71" t="n">
+        <v>805.58</v>
+      </c>
+      <c r="J71" t="n">
+        <v>667.99</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>4070</v>
       </c>
     </row>
     <row r="72">
@@ -2394,11 +3060,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>又见春</t>
+          <t>一李达康一</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>100654578</v>
+        <v>122059844</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -2410,11 +3076,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>和事佬</t>
+          <t>莫桑比克</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>100391957</v>
+        <v>118826076</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -2426,35 +3092,14 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>布小丁</t>
+          <t>洋芋折耳根</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>100116626</v>
-      </c>
-      <c r="D74" t="n">
-        <v>30.15</v>
-      </c>
-      <c r="E74" t="n">
-        <v>1017.75</v>
-      </c>
-      <c r="F74" t="n">
-        <v>894.52</v>
-      </c>
-      <c r="G74" t="n">
-        <v>830.88</v>
-      </c>
-      <c r="H74" t="n">
-        <v>857.28</v>
-      </c>
-      <c r="I74" t="n">
-        <v>854.9299999999999</v>
-      </c>
-      <c r="J74" t="n">
-        <v>670.52</v>
+        <v>118297055</v>
       </c>
       <c r="K74" t="n">
-        <v>5126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2463,11 +3108,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>嘉嘉嘉</t>
+          <t>听雨眠</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>99678853</v>
+        <v>117992119</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -2479,11 +3124,14 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>哇唧唧哇</t>
+          <t>锦衣卫金蝉子</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>99397935</v>
+        <v>116188284</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2492,11 +3140,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>咿呀呀嘿</t>
+          <t>零壹贰壹</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>98248507</v>
+        <v>111853555</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -2508,35 +3156,14 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>爱吃羊肉</t>
+          <t>一匹天涯的马</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>97473105</v>
-      </c>
-      <c r="D78" t="n">
-        <v>29.72</v>
-      </c>
-      <c r="E78" t="n">
-        <v>857</v>
-      </c>
-      <c r="F78" t="n">
-        <v>840</v>
-      </c>
-      <c r="G78" t="n">
-        <v>818</v>
-      </c>
-      <c r="H78" t="n">
-        <v>789</v>
-      </c>
-      <c r="I78" t="n">
-        <v>800</v>
-      </c>
-      <c r="J78" t="n">
-        <v>792</v>
+        <v>110108327</v>
       </c>
       <c r="K78" t="n">
-        <v>4896</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2545,11 +3172,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>叶落落</t>
+          <t>传龙天下</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>97422939</v>
+        <v>109978751</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -2561,11 +3188,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>西点啊</t>
+          <t>秋刀齐爽</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>96935146</v>
+        <v>109628070</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -2577,11 +3204,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>天天骑奉孝夫人</t>
+          <t>月泠瑶</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>96072613</v>
+        <v>108840139</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -2593,35 +3220,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>爱吃肉的棒同学</t>
+          <t>消失的眼袋</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>96025973</v>
-      </c>
-      <c r="D82" t="n">
-        <v>29.06</v>
-      </c>
-      <c r="E82" t="n">
-        <v>907.36</v>
-      </c>
-      <c r="F82" t="n">
-        <v>884.8200000000001</v>
-      </c>
-      <c r="G82" t="n">
-        <v>768.45</v>
-      </c>
-      <c r="H82" t="n">
-        <v>792.75</v>
-      </c>
-      <c r="I82" t="n">
-        <v>736.53</v>
-      </c>
-      <c r="J82" t="n">
-        <v>551.96</v>
+        <v>108094113</v>
       </c>
       <c r="K82" t="n">
-        <v>4642</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -2630,11 +3236,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>舟舟的止水</t>
+          <t>看星星</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>95971354</v>
+        <v>108027627</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -2646,14 +3252,35 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>天马行空</t>
+          <t>玄门丶麟墨</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>95579883</v>
+        <v>105527080</v>
+      </c>
+      <c r="D84" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E84" t="n">
+        <v>968.4299999999999</v>
+      </c>
+      <c r="F84" t="n">
+        <v>915.05</v>
+      </c>
+      <c r="G84" t="n">
+        <v>832.4299999999999</v>
+      </c>
+      <c r="H84" t="n">
+        <v>875.08</v>
+      </c>
+      <c r="I84" t="n">
+        <v>842.11</v>
+      </c>
+      <c r="J84" t="n">
+        <v>694.46</v>
       </c>
       <c r="K84" t="n">
-        <v>0</v>
+        <v>5128</v>
       </c>
     </row>
     <row r="85">
@@ -2662,35 +3289,35 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>扁豆焖面</t>
+          <t>龙吟天下</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>95033759</v>
+        <v>104441967</v>
       </c>
       <c r="D85" t="n">
-        <v>30.48</v>
+        <v>29.2</v>
       </c>
       <c r="E85" t="n">
-        <v>922.26</v>
+        <v>844</v>
       </c>
       <c r="F85" t="n">
-        <v>828.41</v>
+        <v>861</v>
       </c>
       <c r="G85" t="n">
-        <v>762.1</v>
+        <v>683</v>
       </c>
       <c r="H85" t="n">
-        <v>838.09</v>
+        <v>926</v>
       </c>
       <c r="I85" t="n">
-        <v>711.13</v>
+        <v>917</v>
       </c>
       <c r="J85" t="n">
-        <v>537.79</v>
+        <v>684</v>
       </c>
       <c r="K85" t="n">
-        <v>4600</v>
+        <v>4915</v>
       </c>
     </row>
     <row r="86">
@@ -2699,35 +3326,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>啊霞霞霞</t>
+          <t>与落日道晚安</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>93773887</v>
-      </c>
-      <c r="D86" t="n">
-        <v>27</v>
-      </c>
-      <c r="E86" t="n">
-        <v>948.78</v>
-      </c>
-      <c r="F86" t="n">
-        <v>810.22</v>
-      </c>
-      <c r="G86" t="n">
-        <v>641.73</v>
-      </c>
-      <c r="H86" t="n">
-        <v>777.63</v>
-      </c>
-      <c r="I86" t="n">
-        <v>749.95</v>
-      </c>
-      <c r="J86" t="n">
-        <v>568.64</v>
+        <v>102704381</v>
       </c>
       <c r="K86" t="n">
-        <v>4497</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -2736,11 +3342,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>依旧安然</t>
+          <t>小乔啊</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>93246301</v>
+        <v>101251332</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -2752,11 +3358,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>忘忘大礼包</t>
+          <t>哇唧唧哇</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>91957606</v>
+        <v>99397935</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -2768,35 +3374,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>糖菓児</t>
+          <t>咿呀呀嘿</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>91717455</v>
-      </c>
-      <c r="D89" t="n">
-        <v>29.12</v>
-      </c>
-      <c r="E89" t="n">
-        <v>641.34</v>
-      </c>
-      <c r="F89" t="n">
-        <v>777.33</v>
-      </c>
-      <c r="G89" t="n">
-        <v>596.41</v>
-      </c>
-      <c r="H89" t="n">
-        <v>775.55</v>
-      </c>
-      <c r="I89" t="n">
-        <v>776.76</v>
-      </c>
-      <c r="J89" t="n">
-        <v>621.87</v>
+        <v>98248507</v>
       </c>
       <c r="K89" t="n">
-        <v>4189</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -2805,11 +3390,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>地产最少小号</t>
+          <t>舟舟的止水</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>91209747</v>
+        <v>95971354</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -2821,35 +3406,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>厉害的桃夭</t>
+          <t>天马行空</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>91058618</v>
-      </c>
-      <c r="D91" t="n">
-        <v>29.72</v>
-      </c>
-      <c r="E91" t="n">
-        <v>883.04</v>
-      </c>
-      <c r="F91" t="n">
-        <v>841.23</v>
-      </c>
-      <c r="G91" t="n">
-        <v>848.01</v>
-      </c>
-      <c r="H91" t="n">
-        <v>896.9</v>
-      </c>
-      <c r="I91" t="n">
-        <v>779.01</v>
-      </c>
-      <c r="J91" t="n">
-        <v>723.8099999999999</v>
+        <v>95579883</v>
       </c>
       <c r="K91" t="n">
-        <v>4972</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -2858,35 +3422,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>寳尐姐</t>
+          <t>忘忘大礼包</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>90692097</v>
-      </c>
-      <c r="D92" t="n">
-        <v>29.72</v>
-      </c>
-      <c r="E92" t="n">
-        <v>950.7</v>
-      </c>
-      <c r="F92" t="n">
-        <v>778.28</v>
-      </c>
-      <c r="G92" t="n">
-        <v>764.645</v>
-      </c>
-      <c r="H92" t="n">
-        <v>760.28</v>
-      </c>
-      <c r="I92" t="n">
-        <v>752.12</v>
-      </c>
-      <c r="J92" t="n">
-        <v>749.7</v>
+        <v>91957606</v>
       </c>
       <c r="K92" t="n">
-        <v>4756</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -2934,53 +3477,6 @@
         <v>50879805</v>
       </c>
       <c r="K95" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>小怪兽</t>
-        </is>
-      </c>
-      <c r="D96" t="n">
-        <v>29.06</v>
-      </c>
-      <c r="E96" t="n">
-        <v>899.62</v>
-      </c>
-      <c r="F96" t="n">
-        <v>858.49</v>
-      </c>
-      <c r="G96" t="n">
-        <v>716.33</v>
-      </c>
-      <c r="H96" t="n">
-        <v>790.1900000000001</v>
-      </c>
-      <c r="I96" t="n">
-        <v>805.58</v>
-      </c>
-      <c r="J96" t="n">
-        <v>667.99</v>
-      </c>
-      <c r="K96" t="n">
-        <v>4738</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>急急如律令</t>
-        </is>
-      </c>
-      <c r="K97" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>